<commit_message>
Add inline approximate cost columns to capability matrix
</commit_message>
<xml_diff>
--- a/documents/Floater_Capability_Cost_Comparison.xlsx
+++ b/documents/Floater_Capability_Cost_Comparison.xlsx
@@ -45,7 +45,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,16 +94,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -484,12 +492,14 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Offshore Floater Comparison — Capability Matrix</t>
+          <t>Offshore Floater Comparison — Capability &amp; Approximate Cost</t>
         </is>
       </c>
     </row>
@@ -534,395 +544,502 @@
           <t>Best-fit role</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Approx. newbuild CAPEX</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Approx. day-rate / OPEX</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>MPSS (multi-purpose semi-sub)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Deep -&gt; ultra-deep (Sov. Explorer moor rated 600-&gt;1700 m)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Moored or DP</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Yes (combined)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Yes (combined)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>No (offload / pipe)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Good (low heave, column-stabilised)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Combined drill + produce + dive / accommodation on one hull</t>
         </is>
       </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>~$1-2 B modern equiv. (Sov. Explorer GBP 160 M, 1989)</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Field-specific; Balmoral ~GBP 40 M/yr opex</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Drilling semi-sub (MODU)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Mid -&gt; ultra-deep (to ~3,600 m)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Moored / DP2-3</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Very good</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Development &amp; exploration drilling</t>
         </is>
       </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>~$500-750 M</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>~$200-400 k / day</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Drillship</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Ultra-deep (to ~3,600 m+)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>DP3</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Yes (high)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Some (risers / mud)</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Fair (more heave than semi)</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Deepwater drilling, high transit speed, big variable load</t>
         </is>
       </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>~$650 M-$1 B</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>~$300-550 k / day</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Semi-sub FPU / FPV (Balmoral type)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Deep -&gt; ultra-deep</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Moored (or DP)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Limited / none</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>No (export by pipe / shuttle)</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Very good</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Production hub over subsea wells</t>
         </is>
       </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>~$1-2 B modern (Balmoral FPV GBP 160 M, 1989)</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Field-specific opex</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>FPSO</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Shallow -&gt; ultra-deep</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Turret-moored / spread / DP</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>No (usually)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Yes (high)</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Yes (large, 1-2 M bbl)</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Poorer (ship-shape, more heave / roll)</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Remote fields w/o pipeline; storage + offload</t>
         </is>
       </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>~$1-3 B+</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Often leased; opex $100-300 M / yr scale</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Spar</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Deep -&gt; ultra-deep (to ~2,400 m)</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Taut / catenary moored</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Yes (dry trees)</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Excellent (deep-draft, minimal heave)</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Dry-tree production in deepwater</t>
         </is>
       </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>~$1-2 B (hull + topsides)</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Field-specific</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>TLP</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Deep (~1,500 m practical)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Vertical tendons</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Yes (dry trees)</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Excellent vertical (near-zero heave)</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Dry-tree production, direct well access</t>
         </is>
       </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>~$1-2 B</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Field-specific</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>FLNG</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Deep -&gt; ultra-deep</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Turret-moored</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Yes + liquefaction</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Yes (LNG / LPG / condensate)</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Ship-shape, motion-sensitive process</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Stranded gas: liquefy + store + offload</t>
         </is>
       </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>~$2-12 B+ (Prelude ~$12 B+)</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Multi-$100 M / yr</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Jack-up</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Shallow (&lt;= ~150 m)</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Bottom-founded (not a floater in operation)</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Some (production jack-ups)</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>N/A (fixed when jacked)</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Shallow-water drilling / workover</t>
         </is>
       </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>~$180-250 M</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>~$60-150 k / day</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Highlighted rows = MPSS / FPV, the multi-purpose semi concept central to the Lang-Carelli fax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Cost columns (green headers) are order-of-magnitude ballparks; historical GBP values are 1989 figures from the fax, not audited.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -956,14 +1073,14 @@
           <t>Floater</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Newbuild CAPEX</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Day rate / OPEX proxy</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Approx. newbuild CAPEX</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Approx. day rate / OPEX proxy</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -973,197 +1090,197 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>MPSS / FPV (historical, 1989)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Sovereign Explorer GBP 80 M bid -&gt; 160 M final; Balmoral FPV GBP 125 M -&gt; 160 M; Balmoral total field dev GBP 420 M</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Balmoral GBP 40 M / yr opex</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>'Too small for the job - sized to fit the drydock.' Intermingled disciplines made overruns 'uncontrollable.'</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Drilling semi (modern)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>~$500-750 M</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>~$200-400 k / day</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Cyclical; peaks far higher</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Drillship (7th gen)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>~$650 M-$1 B</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>~$300-550 k / day</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Highest variable deckload</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>FPSO</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>~$1-3 B+</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Often leased; opex $100-300 M / yr scale</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Cost driven by topsides &amp; storage size</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Spar</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>~$1-2 B (hull + topsides)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Field-specific</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Deep-draft hull premium</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>TLP</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>~$1-2 B</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Field-specific</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Tendon system cost-sensitive to depth</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>FLNG</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>~$2-12 B+ (Prelude ~$12 B+)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Multi-$100 M / yr</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Most capital-intensive floater class</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Jack-up</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>~$180-250 M</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>~$60-150 k / day</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Shallow-water only</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Figures are order-of-magnitude industry ballparks, not quotes. Historical GBP values are from the 1989 Lang-Carelli fax and are the author's recollection.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>SCRS is not a single standardized industry acronym; here it is read as a self-contained riser &amp; station-keeping/mooring system tied to the MPSS concept.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Ultra-deepwater prize (pre-salt Brazil/Petrobras, GoM, W. Africa) is why multi-purpose semis + self-contained riser/mooring systems were 'keys to trillions.'</t>
         </is>

</xml_diff>

<commit_message>
Correct MPSS row: Lang's deep-draft dry-tree semi-FPU, not Sovereign Explorer
</commit_message>
<xml_diff>
--- a/documents/Floater_Capability_Cost_Comparison.xlsx
+++ b/documents/Floater_Capability_Cost_Comparison.xlsx
@@ -45,7 +45,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,6 +112,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -481,19 +492,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,12 +542,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Hydrocarbon storage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Motion behaviour</t>
+          <t>Tree type / motion</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -558,69 +569,69 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>MPSS (multi-purpose semi-sub)</t>
+          <t>MPSS — Lang's Deep-Draft Dry-Tree Semi-FPU (incl. storage)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Deep -&gt; ultra-deep (Sov. Explorer moor rated 600-&gt;1700 m)</t>
+          <t>Deep -&gt; ultra-deep</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Moored or DP</t>
+          <t>Moored (small-footprint mooring); SCR-capable</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Yes (combined)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Yes (combined)</t>
+          <t>Yes (field-proven)</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>No (offload / pipe)</t>
+          <t>Yes — INCLUDES STORAGE (rare for a semi)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Good (low heave, column-stabilised)</t>
+          <t>Dry tree; deep-draft = excellent (minimal heave)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Combined drill + produce + dive / accommodation on one hull</t>
+          <t>Combined production + drilling + storage with dry trees on a deep-draft semi; built-to-mission</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>~$1-2 B modern equiv. (Sov. Explorer GBP 160 M, 1989)</t>
+          <t>TBD — proprietary concept (Copyright 1984, registered 1987); not costed as a Sovereign-Explorer semi</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Field-specific; Balmoral ~GBP 40 M/yr opex</t>
+          <t>TBD — field-specific</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Drilling semi-sub (MODU)</t>
+          <t>Conventional drilling semi — e.g. Sovereign Explorer (cautionary, 1989)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Mid -&gt; ultra-deep (to ~3,600 m)</t>
+          <t>Deep (moor rated 600 -&gt; later 1000/1700 m)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Moored / DP2-3</t>
+          <t>Moored / DP</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -640,400 +651,459 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Very good</t>
+          <t>Wet tree; good (column-stabilised)</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Development &amp; exploration drilling</t>
+          <t>One-off complex drilling semi built-to-drydock; the fax's cautionary example, NOT an MPSS</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>~$500-750 M</t>
+          <t>GBP 80 M bid -&gt; 160 M final (1989) — ~100% overrun</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>~$200-400 k / day</t>
+          <t>n/a (drilling MODU)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>Semi-sub FPU / FPV — e.g. Balmoral (cautionary, 1989)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Deep -&gt; ultra-deep</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Moored (or DP)</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Limited / none</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>No (export by pipe / shuttle)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Wet tree; very good</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Production hub over subsea wells; Balmoral was undersized 'to fit the drydock'</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GBP 125 M -&gt; 160 M (1989); Balmoral total field dev GBP 420 M</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Balmoral ~GBP 40 M / yr opex</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Drilling semi-sub (MODU, modern)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Mid -&gt; ultra-deep (to ~3,600 m)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Moored / DP2-3</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Wet tree; very good</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Development &amp; exploration drilling</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>~$500-750 M</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>~$200-400 k / day</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t>Drillship</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Ultra-deep (to ~3,600 m+)</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>DP3</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Yes (high)</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Some (risers / mud)</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>Fair (more heave than semi)</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Wet tree; fair (more heave than semi)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Deepwater drilling, high transit speed, big variable load</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>~$650 M-$1 B</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>~$300-550 k / day</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Semi-sub FPU / FPV (Balmoral type)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>FPSO</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Shallow -&gt; ultra-deep</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Turret / spread moored / DP</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>No (usually)</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Yes (high)</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Yes (large, 1-2 M bbl)</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Wet tree; poorer (ship-shape heave/roll)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Remote fields w/o pipeline; storage + offload</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>~$1-3 B+</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Often leased; opex $100-300 M / yr scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Spar</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Deep -&gt; ultra-deep (to ~2,400 m)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Taut / catenary moored</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Yes (dry trees)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Limited</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Dry tree; excellent (deep-draft, minimal heave)</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Dry-tree production in deepwater</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>~$1-2 B (hull + topsides)</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Field-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>TLP</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Deep (~1,500 m practical)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Vertical tendons</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Yes (dry trees)</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Dry tree; excellent vertical (near-zero heave)</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Dry-tree production, direct well access</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>~$1-2 B</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Field-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>FLNG</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Deep -&gt; ultra-deep</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Moored (or DP)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Limited / none</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Turret-moored</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Yes + liquefaction</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Yes (LNG / LPG / condensate)</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Ship-shape; motion-sensitive process</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Stranded gas: liquefy + store + offload</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>~$2-12 B+ (Prelude ~$12 B+)</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Multi-$100 M / yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Jack-up</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Shallow (&lt;= ~150 m)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Bottom-founded (not floating in operation)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>No (export by pipe / shuttle)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Very good</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Production hub over subsea wells</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>~$1-2 B modern (Balmoral FPV GBP 160 M, 1989)</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Field-specific opex</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>FPSO</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Shallow -&gt; ultra-deep</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Turret-moored / spread / DP</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>No (usually)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Yes (high)</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Yes (large, 1-2 M bbl)</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Poorer (ship-shape, more heave / roll)</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Remote fields w/o pipeline; storage + offload</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>~$1-3 B+</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>Often leased; opex $100-300 M / yr scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Spar</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Deep -&gt; ultra-deep (to ~2,400 m)</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Taut / catenary moored</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Yes (dry trees)</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Limited</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Excellent (deep-draft, minimal heave)</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Dry-tree production in deepwater</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>~$1-2 B (hull + topsides)</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Field-specific</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>TLP</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Deep (~1,500 m practical)</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Vertical tendons</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Yes (dry trees)</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Some (production jack-ups)</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Excellent vertical (near-zero heave)</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>Dry-tree production, direct well access</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>~$1-2 B</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Field-specific</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>FLNG</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Deep -&gt; ultra-deep</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Turret-moored</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Yes + liquefaction</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Yes (LNG / LPG / condensate)</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Ship-shape, motion-sensitive process</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Stranded gas: liquefy + store + offload</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>~$2-12 B+ (Prelude ~$12 B+)</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Multi-$100 M / yr</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Jack-up</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Shallow (&lt;= ~150 m)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Bottom-founded (not a floater in operation)</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Some (production jack-ups)</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>N/A (fixed when jacked)</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Fixed when jacked</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Shallow-water drilling / workover</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>~$180-250 M</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J13" s="9" t="inlineStr">
         <is>
           <t>~$60-150 k / day</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Highlighted rows = MPSS / FPV, the multi-purpose semi concept central to the Lang-Carelli fax.</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Cost columns (green headers) are order-of-magnitude ballparks; historical GBP values are 1989 figures from the fax, not audited.</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Orange row = MPSS (Lang's registered Deep-Draft Dry-Tree Semi-FPU, incl. storage). Yellow rows = 1989 cautionary examples from the Lang-Carelli fax — conventional units, NOT MPSS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>MPSS row per Wood Group Mustang 'Deepwater Concept Selection Matrix' (Semi-FPU / Deep Draft Dry Tree). SCR = Steel Catenary Riser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Cost columns (green headers) are order-of-magnitude ballparks; historical GBP values are 1989 figures from the fax, not audited. MPSS build cost intentionally TBD, not equated to Sovereign Explorer.</t>
         </is>
       </c>
     </row>
@@ -1051,13 +1121,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1092,197 +1162,241 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>MPSS / FPV (historical, 1989)</t>
+          <t>MPSS — Lang's Deep-Draft Dry-Tree Semi-FPU</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Sovereign Explorer GBP 80 M bid -&gt; 160 M final; Balmoral FPV GBP 125 M -&gt; 160 M; Balmoral total field dev GBP 420 M</t>
+          <t>TBD — proprietary concept (Copyright 1984, Certificate of Registration 30 Oct 1987)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Balmoral GBP 40 M / yr opex</t>
+          <t>TBD — field-specific</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>'Too small for the job - sized to fit the drydock.' Intermingled disciplines made overruns 'uncontrollable.'</t>
+          <t>Deep-draft dry-tree semi that INCLUDES STORAGE. Distinct from the Sovereign Explorer. Concept per Wood Group Mustang selection matrix.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Drilling semi (modern)</t>
+          <t>Conventional drilling semi — Sovereign Explorer (1989, cautionary)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>~$500-750 M</t>
+          <t>GBP 80 M bid -&gt; 160 M final (~100% overrun)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>~$200-400 k / day</t>
+          <t>n/a (drilling MODU)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Cyclical; peaks far higher</t>
+          <t>First semi for the yard; combined chain+cable mooring, derrick 500-&gt;700te. 'Too small... sized to fit the drydock.' NOT an MPSS.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>Semi-sub FPV — Balmoral (1989, cautionary)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>GBP 125 M -&gt; 160 M; Balmoral total field dev GBP 420 M</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Balmoral GBP 40 M / yr opex; +0.7% ROI at 40,000 bbls/day</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Undersized to fit existing drydocks; intermingled disciplines made overruns 'uncontrollable.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Drilling semi (modern)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>~$500-750 M</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>~$200-400 k / day</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Cyclical; peaks far higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t>Drillship (7th gen)</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>~$650 M-$1 B</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>~$300-550 k / day</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Highest variable deckload</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>FPSO</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>~$1-3 B+</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Often leased; opex $100-300 M / yr scale</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Cost driven by topsides &amp; storage size</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Spar</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>~$1-2 B (hull + topsides)</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Field-specific</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Deep-draft hull premium</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>TLP</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>~$1-2 B</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Field-specific</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Tendon system cost-sensitive to depth</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>FLNG</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>~$2-12 B+ (Prelude ~$12 B+)</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Multi-$100 M / yr</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Most capital-intensive floater class</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Jack-up</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>~$180-250 M</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>~$60-150 k / day</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Shallow-water only</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Figures are order-of-magnitude industry ballparks, not quotes. Historical GBP values are from the 1989 Lang-Carelli fax and are the author's recollection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>SCRS is not a single standardized industry acronym; here it is read as a self-contained riser &amp; station-keeping/mooring system tied to the MPSS concept.</t>
+          <t>Jack-up</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>~$180-250 M</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>~$60-150 k / day</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Shallow-water only</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Ultra-deepwater prize (pre-salt Brazil/Petrobras, GoM, W. Africa) is why multi-purpose semis + self-contained riser/mooring systems were 'keys to trillions.'</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Figures are order-of-magnitude industry ballparks, not quotes. Historical GBP values are from the 1989 Lang-Carelli fax (author's recollection).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>MPSS = Lang's Multi-Purpose Semi-Submersible: a Deep-Draft Dry-Tree Semi-FPU that includes storage. It is NOT the Sovereign Explorer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>SCR = Steel Catenary Riser. MPSS + steel catenary risers were the enabling pairing for ultra-deepwater tiebacks (pre-salt Brazil/Petrobras, GoM, W. Africa).</t>
         </is>
       </c>
     </row>

</xml_diff>